<commit_message>
correccion excel, ajuste time cell y add templates
</commit_message>
<xml_diff>
--- a/exports/templates/importacion/template_importacion_horarios_minimo.xlsx
+++ b/exports/templates/importacion/template_importacion_horarios_minimo.xlsx
@@ -5,13 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Modulos" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Guia" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Sem1" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="31">
   <si>
     <t>ID Clase</t>
   </si>
@@ -28,23 +30,89 @@
     <t>Lunes</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>FIS-201</t>
+  </si>
+  <si>
+    <t>Martes</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Template: Importacion horarios (Minimo)</t>
+  </si>
+  <si>
+    <t>Tipo importacion: IMPORTAR DATOS UNICOS &gt; horarios</t>
+  </si>
+  <si>
+    <t>Perfil: MINIMO</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>Este template incluye solo columnas obligatorias.</t>
+  </si>
+  <si>
+    <t>Importante</t>
+  </si>
+  <si>
+    <t>Las columnas opcionales solo se importan si tienen datos.</t>
+  </si>
+  <si>
+    <t>Campo</t>
+  </si>
+  <si>
+    <t>Uso</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Codigo unico del grupo</t>
+  </si>
+  <si>
+    <t>Obligatorio</t>
+  </si>
+  <si>
+    <t>Dia del horario. Ej: Lunes</t>
+  </si>
+  <si>
+    <t>Modulo del horario. Ej: 1</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>Miercoles</t>
   </si>
   <si>
-    <t>FIS-201</t>
-  </si>
-  <si>
-    <t>Martes</t>
-  </si>
-  <si>
     <t>Jueves</t>
+  </si>
+  <si>
+    <t>Viernes</t>
+  </si>
+  <si>
+    <t>08:00-09:30</t>
+  </si>
+  <si>
+    <t>N de clase INF-101</t>
+  </si>
+  <si>
+    <t>09:30-11:00</t>
+  </si>
+  <si>
+    <t>N de clase FIS-201</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -54,17 +122,31 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -72,13 +154,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,15 +514,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="1" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -444,41 +538,185 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
-        <v>1</v>
+      <c r="C2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="56" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="B10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="6" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5">
-        <v>3</v>
+      <c r="D1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>